<commit_message>
feat: de-fragilize PCR reads and provider week/year; weekly run artifacts
Pipeline robustness (docs/TODO.md architecture items):
- PCR: list.files now filters to .xls/.xlsx, ignoring the .eds export
- wnv_s_clean(): add force_recompute arg to re-derive week+year from
  trap_date on raw provider input; default FALSE preserves the historical
  read-back gate
- wire force_recompute=TRUE at the datasheet and all_species call sites
- clean_4_weekly_input(): derive Year from Trap Date so a stale provider
  year no longer drops samples into non_week_samples.csv
- tests: source wnv_s_clean in helper-setup, add test-clean_wnv_s.R
- README: fix stale pipeline filename, nav list, step numbering, flags

Also includes this week's (2026 w24) run artifacts.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/1_input/2026/w24/datasheet/08JuneWNV 2026 BC Data Sheet.xlsx
+++ b/1_input/2026/w24/datasheet/08JuneWNV 2026 BC Data Sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Programming_Directory/Ebel_Lab/wnv-ss-wkly_report/1_input/2026/w24/datasheet/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft11751656.sharepoint.com/sites/TL/Shared Documents/Projects/City of Boulder - Mosquito Project/2026/Adults/Week 4 (08June2026)/WNV testing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C1AC080-AE6D-E645-88B3-4D1AE6BAB7DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{57982CC1-E383-4C71-81D1-2E658D5161F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DEF43DF-9094-4D39-ADCE-1C26E64BDFBC}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="20740" windowHeight="11160" xr2:uid="{4D1E2C8E-A4DF-4A6D-8027-4BABF8155C5C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{4D1E2C8E-A4DF-4A6D-8027-4BABF8155C5C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -159,7 +159,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -596,15 +596,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C2ADBAF-23C3-4467-80DC-4743B39CFDBB}">
   <dimension ref="A1:S6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="18" max="18" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.5" customWidth="1"/>
+    <col min="18" max="18" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="71" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" ht="64.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -663,7 +663,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" ht="15.75" customHeight="1">
       <c r="A2" s="9">
         <v>2026</v>
       </c>
@@ -672,7 +672,7 @@
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="6">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="E2" s="7">
         <v>46181</v>
@@ -714,7 +714,7 @@
       <c r="R2" s="5"/>
       <c r="S2" s="8"/>
     </row>
-    <row r="3" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" ht="15.75" customHeight="1">
       <c r="A3" s="9">
         <v>2026</v>
       </c>
@@ -723,7 +723,7 @@
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="6">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="E3" s="7">
         <v>46181</v>
@@ -765,7 +765,7 @@
       <c r="R3" s="5"/>
       <c r="S3" s="8"/>
     </row>
-    <row r="4" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" ht="15.75" customHeight="1">
       <c r="A4" s="9">
         <v>2026</v>
       </c>
@@ -774,7 +774,7 @@
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="6">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="E4" s="7">
         <v>46181</v>
@@ -816,7 +816,7 @@
       <c r="R4" s="5"/>
       <c r="S4" s="8"/>
     </row>
-    <row r="5" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:19" ht="15.75" customHeight="1">
       <c r="A5" s="9">
         <v>2026</v>
       </c>
@@ -825,7 +825,7 @@
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="6">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="E5" s="7">
         <v>46181</v>
@@ -867,7 +867,7 @@
       <c r="R5" s="5"/>
       <c r="S5" s="8"/>
     </row>
-    <row r="6" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:19" ht="15.75" customHeight="1">
       <c r="A6" s="9">
         <v>2026</v>
       </c>
@@ -876,7 +876,7 @@
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="6">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="E6" s="7">
         <v>46181</v>
@@ -936,6 +936,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A700E0BBAD20834882D4451FE2A4028E" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="646ac923dc796cd605cd3f4a990e63ec">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6aff204b-29f3-4740-958e-d447a0231527" xmlns:ns3="68ae4a9d-1816-47aa-9ee7-1576dec6189d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4235439834c5878493508215d82d9fde" ns2:_="" ns3:_="">
     <xsd:import namespace="6aff204b-29f3-4740-958e-d447a0231527"/>
@@ -1148,15 +1157,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3490C7FC-DFD1-4D03-9E83-7BB698782D79}">
   <ds:schemaRefs>
@@ -1169,6 +1169,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{10106931-061F-44D8-A931-4F6EC49BD08B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BA239FF-650C-4ACD-8320-043F6ACDE59D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1185,12 +1193,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{10106931-061F-44D8-A931-4F6EC49BD08B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>